<commit_message>
♻️ refactor: remove direct organization relation, use customer.organization instead
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/NomadDocs/Completed Work Certificates.xlsx
+++ b/apps/excel-service/templates/NomadDocs/Completed Work Certificates.xlsx
@@ -162,10 +162,10 @@
     <t xml:space="preserve">Дата подписания (принятия) работ (услуг)</t>
   </si>
   <si>
-    <t xml:space="preserve">{organization.organization}, город {organization.city}, {organization.index}, {organization.address}</t>
-  </si>
-  <si>
-    <t>{organization.bin}</t>
+    <t xml:space="preserve">{customer.organization.organization}, город {customer.organization.city}, {customer.organization.index}, {customer.organization.address}</t>
+  </si>
+  <si>
+    <t>{customer.organization.bin}</t>
   </si>
   <si>
     <t xml:space="preserve">Индивидуальный предприниматель «NomadDocs»  Жалтырбаев Әділет Ғалымұлы                                                                               Карагандинская область, г. Караганда,район имени Казыбек Би, улица Гапеева, дом 15/1, блок Б, квартира №101</t>

</xml_diff>